<commit_message>
biomedy i costam 2.0
</commit_message>
<xml_diff>
--- a/Semestr 4/Cad/2ME-PCBLAB/Michal_Wojna/Lab_4_schematic/tabela_impedancji.xlsx
+++ b/Semestr 4/Cad/2ME-PCBLAB/Michal_Wojna/Lab_4_schematic/tabela_impedancji.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\Desktop\Git\aghmtm\Semestr 4\Cad\2ME-PCBLAB\Michal_Wojna\Lab_4_schematic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF506A6-9D10-4242-BE36-B364621D12FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F56AEF6-B865-44A5-815B-2855CA6C6132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="13583" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zestawienie Impedancji" sheetId="1" r:id="rId1"/>
@@ -65,13 +65,13 @@
 1mm</t>
   </si>
   <si>
-    <t>154Ω</t>
-  </si>
-  <si>
-    <t>159Ω</t>
-  </si>
-  <si>
-    <t>158Ω</t>
+    <t>79.4Ω</t>
+  </si>
+  <si>
+    <t>102Ω</t>
+  </si>
+  <si>
+    <t>111Ω</t>
   </si>
 </sst>
 </file>

</xml_diff>